<commit_message>
R7: compute real NAV / P&L / benchmark in reporting (no hard-coded zeros)
- Reporting node fetches current prices (held symbols + SPY) via market_data
  and passes them to the agent (agent stays IO-free)
- NAV = cash + Σ(qty×price); unrealized P&L = Σ((price−avg_cost)×qty);
  benchmark_return = SPY day return; positions carry current_price + unrealized_pnl
- demo Summary shows computed NAV=100000, benchmark=0.2153% (was hard-coded 0)
- suite green (276)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/2024-10-23.xlsx
+++ b/reports/2024-10-23.xlsx
@@ -468,10 +468,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.002152574479076976</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>-0.002152574479076976</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>